<commit_message>
v1.0.2 Add single ended
</commit_message>
<xml_diff>
--- a/database/line_data.xlsx
+++ b/database/line_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fault-locator-app\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54E7906C-2527-4407-9808-A3F4DCDE07A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE0B172C-08A4-4E15-8BC8-95568D728E95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -837,8 +837,8 @@
         <v>1.697758643771252</v>
       </c>
       <c r="O3" s="6">
-        <f>IMARGUMENT(M3)</f>
-        <v>1.2583869429820267</v>
+        <f>DEGREES(IMARGUMENT(M3))</f>
+        <v>72.100260827239893</v>
       </c>
       <c r="P3" s="7" t="s">
         <v>17</v>
@@ -908,8 +908,8 @@
         <v>1.697758643771252</v>
       </c>
       <c r="O4" s="6">
-        <f t="shared" ref="O4:O24" si="5">IMARGUMENT(M4)</f>
-        <v>1.2583869429820267</v>
+        <f t="shared" ref="O4:O24" si="5">DEGREES(IMARGUMENT(M4))</f>
+        <v>72.100260827239893</v>
       </c>
       <c r="P4" s="7" t="s">
         <v>17</v>
@@ -980,7 +980,7 @@
       </c>
       <c r="O5" s="6">
         <f t="shared" si="5"/>
-        <v>1.2583869429820267</v>
+        <v>72.100260827239893</v>
       </c>
       <c r="P5" s="7" t="s">
         <v>17</v>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="O6" s="6">
         <f t="shared" si="5"/>
-        <v>1.2583869429820267</v>
+        <v>72.100260827239893</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>34</v>
@@ -1121,8 +1121,8 @@
         <v>1.697758643771252</v>
       </c>
       <c r="O7" s="6">
-        <f t="shared" ref="O7:O8" si="11">IMARGUMENT(M7)</f>
-        <v>1.2583869429820267</v>
+        <f t="shared" si="5"/>
+        <v>72.100260827239893</v>
       </c>
       <c r="P7" s="7" t="s">
         <v>36</v>
@@ -1192,8 +1192,8 @@
         <v>1.4966147566090613</v>
       </c>
       <c r="O8" s="6">
-        <f t="shared" si="11"/>
-        <v>1.2599509424940258</v>
+        <f t="shared" si="5"/>
+        <v>72.189871398437973</v>
       </c>
       <c r="P8" s="7" t="s">
         <v>38</v>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="O9" s="6">
         <f t="shared" si="5"/>
-        <v>1.2599509424940258</v>
+        <v>72.189871398437973</v>
       </c>
       <c r="P9" s="7" t="s">
         <v>38</v>
@@ -1326,7 +1326,7 @@
         <v>1.61558</v>
       </c>
       <c r="M10" s="6" t="str">
-        <f t="shared" ref="M10" si="12">COMPLEX(K10,L10)</f>
+        <f t="shared" ref="M10" si="11">COMPLEX(K10,L10)</f>
         <v>0,52181+1,61558i</v>
       </c>
       <c r="N10" s="6">
@@ -1334,8 +1334,8 @@
         <v>1.697758643771252</v>
       </c>
       <c r="O10" s="6">
-        <f t="shared" ref="O10" si="13">IMARGUMENT(M10)</f>
-        <v>1.2583869429820267</v>
+        <f t="shared" si="5"/>
+        <v>72.100260827239893</v>
       </c>
       <c r="P10" s="7" t="s">
         <v>36</v>
@@ -1379,11 +1379,11 @@
         <v>0.42399999999999999</v>
       </c>
       <c r="H11" s="4" t="str">
-        <f t="shared" ref="H11:H14" si="14">COMPLEX(F11,G11)</f>
+        <f t="shared" ref="H11:H14" si="12">COMPLEX(F11,G11)</f>
         <v>0,128+0,424i</v>
       </c>
       <c r="I11" s="2">
-        <f t="shared" ref="I11:I14" si="15">IMABS(H11)</f>
+        <f t="shared" ref="I11:I14" si="13">IMABS(H11)</f>
         <v>0.44289953714132513</v>
       </c>
       <c r="J11" s="2">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="O11" s="6">
         <f t="shared" si="5"/>
-        <v>1.2583869429820267</v>
+        <v>72.100260827239893</v>
       </c>
       <c r="P11" s="7" t="s">
         <v>36</v>
@@ -1450,11 +1450,11 @@
         <v>0.23358999999999999</v>
       </c>
       <c r="H12" s="4" t="str">
-        <f t="shared" ref="H12" si="16">COMPLEX(F12,G12)</f>
+        <f t="shared" ref="H12" si="14">COMPLEX(F12,G12)</f>
         <v>0,04903+0,23359i</v>
       </c>
       <c r="I12" s="2">
-        <f t="shared" ref="I12" si="17">IMABS(H12)</f>
+        <f t="shared" ref="I12" si="15">IMABS(H12)</f>
         <v>0.23868018141437716</v>
       </c>
       <c r="J12" s="2">
@@ -1468,7 +1468,7 @@
         <v>1.42489</v>
       </c>
       <c r="M12" s="6" t="str">
-        <f t="shared" ref="M12" si="18">COMPLEX(K12,L12)</f>
+        <f t="shared" ref="M12" si="16">COMPLEX(K12,L12)</f>
         <v>0,45776+1,42489i</v>
       </c>
       <c r="N12" s="6">
@@ -1476,8 +1476,8 @@
         <v>1.4966147566090613</v>
       </c>
       <c r="O12" s="6">
-        <f t="shared" ref="O12" si="19">IMARGUMENT(M12)</f>
-        <v>1.2599509424940258</v>
+        <f t="shared" si="5"/>
+        <v>72.189871398437973</v>
       </c>
       <c r="P12" s="7" t="s">
         <v>38</v>
@@ -1521,11 +1521,11 @@
         <v>0.23358999999999999</v>
       </c>
       <c r="H13" s="4" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0,04903+0,23359i</v>
       </c>
       <c r="I13" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.23868018141437716</v>
       </c>
       <c r="J13" s="2">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="O13" s="6">
         <f t="shared" si="5"/>
-        <v>1.2599509424940258</v>
+        <v>72.189871398437973</v>
       </c>
       <c r="P13" s="7" t="s">
         <v>38</v>
@@ -1592,11 +1592,11 @@
         <v>0.40054000000000001</v>
       </c>
       <c r="H14" s="4" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0,09774+0,40054i</v>
       </c>
       <c r="I14" s="2">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.41229285611079891</v>
       </c>
       <c r="J14" s="2">
@@ -1619,7 +1619,7 @@
       </c>
       <c r="O14" s="6">
         <f t="shared" si="5"/>
-        <v>1.3674735747897941</v>
+        <v>78.350464431122532</v>
       </c>
       <c r="P14" s="7" t="s">
         <v>38</v>
@@ -1663,11 +1663,11 @@
         <v>0.40656999999999999</v>
       </c>
       <c r="H15" s="4" t="str">
-        <f t="shared" ref="H15" si="20">COMPLEX(F15,G15)</f>
+        <f t="shared" ref="H15" si="17">COMPLEX(F15,G15)</f>
         <v>0,09645+0,40657i</v>
       </c>
       <c r="I15" s="2">
-        <f t="shared" ref="I15" si="21">IMABS(H15)</f>
+        <f t="shared" ref="I15" si="18">IMABS(H15)</f>
         <v>0.41785376317558748</v>
       </c>
       <c r="J15" s="2">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="O15" s="6">
         <f t="shared" si="5"/>
-        <v>1.3831522852746667</v>
+        <v>79.248788370113246</v>
       </c>
       <c r="P15" s="7" t="s">
         <v>38</v>
@@ -1734,11 +1734,11 @@
         <v>0.40054000000000001</v>
       </c>
       <c r="H16" s="4" t="str">
-        <f t="shared" ref="H16:H19" si="22">COMPLEX(F16,G16)</f>
+        <f t="shared" ref="H16:H19" si="19">COMPLEX(F16,G16)</f>
         <v>0,09774+0,40054i</v>
       </c>
       <c r="I16" s="2">
-        <f t="shared" ref="I16:I19" si="23">IMABS(H16)</f>
+        <f t="shared" ref="I16:I19" si="20">IMABS(H16)</f>
         <v>0.41229285611079891</v>
       </c>
       <c r="J16" s="2">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="O16" s="6">
         <f t="shared" si="5"/>
-        <v>1.3674735747897941</v>
+        <v>78.350464431122532</v>
       </c>
       <c r="P16" s="7" t="s">
         <v>34</v>
@@ -1805,11 +1805,11 @@
         <v>0.23400000000000001</v>
       </c>
       <c r="H17" s="4" t="str">
-        <f t="shared" ref="H17" si="24">COMPLEX(F17,G17)</f>
+        <f t="shared" ref="H17" si="21">COMPLEX(F17,G17)</f>
         <v>0,064+0,234i</v>
       </c>
       <c r="I17" s="2">
-        <f t="shared" ref="I17" si="25">IMABS(H17)</f>
+        <f t="shared" ref="I17" si="22">IMABS(H17)</f>
         <v>0.24259431155738176</v>
       </c>
       <c r="J17" s="2">
@@ -1823,7 +1823,7 @@
         <v>1.42489</v>
       </c>
       <c r="M17" s="6" t="str">
-        <f t="shared" ref="M17" si="26">COMPLEX(K17,L17)</f>
+        <f t="shared" ref="M17" si="23">COMPLEX(K17,L17)</f>
         <v>0,45776+1,42489i</v>
       </c>
       <c r="N17" s="6">
@@ -1831,8 +1831,8 @@
         <v>1.4966147566090613</v>
       </c>
       <c r="O17" s="6">
-        <f t="shared" ref="O17" si="27">IMARGUMENT(M17)</f>
-        <v>1.2599509424940258</v>
+        <f t="shared" si="5"/>
+        <v>72.189871398437973</v>
       </c>
       <c r="P17" s="7" t="s">
         <v>42</v>
@@ -1876,11 +1876,11 @@
         <v>0.23400000000000001</v>
       </c>
       <c r="H18" s="4" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="19"/>
         <v>0,064+0,234i</v>
       </c>
       <c r="I18" s="2">
-        <f t="shared" si="23"/>
+        <f t="shared" si="20"/>
         <v>0.24259431155738176</v>
       </c>
       <c r="J18" s="2">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="O18" s="6">
         <f t="shared" si="5"/>
-        <v>1.2599509424940258</v>
+        <v>72.189871398437973</v>
       </c>
       <c r="P18" s="7" t="s">
         <v>42</v>
@@ -1947,11 +1947,11 @@
         <v>0.42399999999999999</v>
       </c>
       <c r="H19" s="4" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="19"/>
         <v>0,128+0,424i</v>
       </c>
       <c r="I19" s="2">
-        <f t="shared" si="23"/>
+        <f t="shared" si="20"/>
         <v>0.44289953714132513</v>
       </c>
       <c r="J19" s="2">
@@ -1965,7 +1965,7 @@
         <v>1.61558</v>
       </c>
       <c r="M19" s="6" t="str">
-        <f t="shared" ref="M19" si="28">COMPLEX(K19,L19)</f>
+        <f t="shared" ref="M19" si="24">COMPLEX(K19,L19)</f>
         <v>0,52181+1,61558i</v>
       </c>
       <c r="N19" s="6">
@@ -1973,8 +1973,8 @@
         <v>1.697758643771252</v>
       </c>
       <c r="O19" s="6">
-        <f t="shared" ref="O19" si="29">IMARGUMENT(M19)</f>
-        <v>1.2583869429820267</v>
+        <f t="shared" si="5"/>
+        <v>72.100260827239893</v>
       </c>
       <c r="P19" s="7" t="s">
         <v>38</v>
@@ -2018,11 +2018,11 @@
         <v>0.42399999999999999</v>
       </c>
       <c r="H20" s="4" t="str">
-        <f t="shared" ref="H20:H23" si="30">COMPLEX(F20,G20)</f>
+        <f t="shared" ref="H20:H23" si="25">COMPLEX(F20,G20)</f>
         <v>0,128+0,424i</v>
       </c>
       <c r="I20" s="2">
-        <f t="shared" ref="I20:I23" si="31">IMABS(H20)</f>
+        <f t="shared" ref="I20:I23" si="26">IMABS(H20)</f>
         <v>0.44289953714132513</v>
       </c>
       <c r="J20" s="2">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="5"/>
-        <v>1.2583869429820267</v>
+        <v>72.100260827239893</v>
       </c>
       <c r="P20" s="7" t="s">
         <v>38</v>
@@ -2089,11 +2089,11 @@
         <v>0.23730999999999999</v>
       </c>
       <c r="H21" s="4" t="str">
-        <f t="shared" ref="H21" si="32">COMPLEX(F21,G21)</f>
+        <f t="shared" ref="H21" si="27">COMPLEX(F21,G21)</f>
         <v>0,363+0,23731i</v>
       </c>
       <c r="I21" s="2">
-        <f t="shared" ref="I21" si="33">IMABS(H21)</f>
+        <f t="shared" ref="I21" si="28">IMABS(H21)</f>
         <v>0.43368771725747546</v>
       </c>
       <c r="J21" s="2">
@@ -2107,7 +2107,7 @@
         <v>1.3763099999999999</v>
       </c>
       <c r="M21" s="6" t="str">
-        <f t="shared" ref="M21" si="34">COMPLEX(K21,L21)</f>
+        <f t="shared" ref="M21" si="29">COMPLEX(K21,L21)</f>
         <v>0,38899+1,37631i</v>
       </c>
       <c r="N21" s="6">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="5"/>
-        <v>1.2953481364616168</v>
+        <v>74.217981219386871</v>
       </c>
       <c r="P21" s="7" t="s">
         <v>42</v>
@@ -2160,11 +2160,11 @@
         <v>0.23730999999999999</v>
       </c>
       <c r="H22" s="4" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="25"/>
         <v>0,363+0,23731i</v>
       </c>
       <c r="I22" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="26"/>
         <v>0.43368771725747546</v>
       </c>
       <c r="J22" s="2">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="O22" s="6">
         <f t="shared" si="5"/>
-        <v>1.2953481364616168</v>
+        <v>74.217981219386871</v>
       </c>
       <c r="P22" s="7" t="s">
         <v>42</v>
@@ -2231,11 +2231,11 @@
         <v>0.23730999999999999</v>
       </c>
       <c r="H23" s="4" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="25"/>
         <v>0,363+0,23731i</v>
       </c>
       <c r="I23" s="2">
-        <f t="shared" si="31"/>
+        <f t="shared" si="26"/>
         <v>0.43368771725747546</v>
       </c>
       <c r="J23" s="2">
@@ -2249,7 +2249,7 @@
         <v>1.3763099999999999</v>
       </c>
       <c r="M23" s="6" t="str">
-        <f t="shared" ref="M23" si="35">COMPLEX(K23,L23)</f>
+        <f t="shared" ref="M23" si="30">COMPLEX(K23,L23)</f>
         <v>0,38899+1,37631i</v>
       </c>
       <c r="N23" s="6">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="O23" s="6">
         <f t="shared" si="5"/>
-        <v>1.2953481364616168</v>
+        <v>74.217981219386871</v>
       </c>
       <c r="P23" s="7" t="s">
         <v>42</v>
@@ -2302,11 +2302,11 @@
         <v>0.23730999999999999</v>
       </c>
       <c r="H24" s="4" t="str">
-        <f t="shared" ref="H24" si="36">COMPLEX(F24,G24)</f>
+        <f t="shared" ref="H24" si="31">COMPLEX(F24,G24)</f>
         <v>0,363+0,23731i</v>
       </c>
       <c r="I24" s="2">
-        <f t="shared" ref="I24" si="37">IMABS(H24)</f>
+        <f t="shared" ref="I24" si="32">IMABS(H24)</f>
         <v>0.43368771725747546</v>
       </c>
       <c r="J24" s="2">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="O24" s="6">
         <f t="shared" si="5"/>
-        <v>1.2953481364616168</v>
+        <v>74.217981219386871</v>
       </c>
       <c r="P24" s="7" t="s">
         <v>42</v>

</xml_diff>